<commit_message>
add modify_test automation files_playwrights
</commit_message>
<xml_diff>
--- a/IT23139930/IT23139930.xlsx
+++ b/IT23139930/IT23139930.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eneth\Desktop\IT23139930\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50EF900F-E95E-402F-BD81-BEBC06B9F711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749D06AA-2A6B-4941-851E-CF740E007C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="280">
   <si>
     <t>TC ID</t>
   </si>
@@ -234,9 +234,6 @@
     <t>Pos_Fun_0025</t>
   </si>
   <si>
-    <t>මට එක දෙන්න කරුණාකර. මම එන්න හිතන් ඉන්නේ?</t>
-  </si>
-  <si>
     <t>Pos_Fun_0026</t>
   </si>
   <si>
@@ -255,9 +252,6 @@
     <t>ayubowan machan! suba aluth awurudhak vewe!</t>
   </si>
   <si>
-    <t>අයුබෝවන් මැචන්! සුභ අලුත් අවුරුද්දක් වේවේ</t>
-  </si>
-  <si>
     <t>Pos_Fun_0028</t>
   </si>
   <si>
@@ -408,15 +402,9 @@
     <t>මම ගෙදර යනවා.</t>
   </si>
   <si>
-    <t>&lt;h1&gt; Hello&lt;/h1&gt;</t>
-  </si>
-  <si>
     <t>Pos_Fun_0048</t>
   </si>
   <si>
-    <t>eyaa adha kiyavanavaa vaedi naedhdha. @mata nam ahan i#dhallaa epaa velaa</t>
-  </si>
-  <si>
     <t>එයා අද කියවනවා වැඩි නැද්ද. මට නම් අහන් ඉදලා එපා වෙලා</t>
   </si>
   <si>
@@ -438,12 +426,6 @@
     <t>එපා කියලා මම කියන්නේ නිසා ඔයාට එක තේරුම් ගන්න ඕනි</t>
   </si>
   <si>
-    <t>අපි තම කනවා.</t>
-  </si>
-  <si>
-    <t>api thma kanavaa</t>
-  </si>
-  <si>
     <t>Teams meeting eka link eka WhatsApp karanna</t>
   </si>
   <si>
@@ -453,9 +435,6 @@
     <t>api trip ek Kandy walata yamud traffic nisaa yanakota parakkuwei da?</t>
   </si>
   <si>
-    <t>අපි trip එක් Kandy වලට යමුද traffic නිසා යනකොට පරක්කුවෙයි ද?</t>
-  </si>
-  <si>
     <t>mm ee gaena balaaporoththu thiyagana hitiyaa</t>
   </si>
   <si>
@@ -465,61 +444,24 @@
     <t>marthu masa mata exam ek tiyenawa</t>
   </si>
   <si>
-    <t>මාර්තු මාසේ මට exam එක් තියෙනවා</t>
-  </si>
-  <si>
     <t>hata udee 8.30 ta office yanna enn.</t>
   </si>
   <si>
-    <t>හට උදේ 8.30 ට office යන්න එන්න</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mr. pereeraa, mata ad office enna parakku venavaa. mokadha bus eke godak senaga , hodhatama traffic baththaramulla hatiyee. meeting eka patan ganna kalin mama enavaa. mata documents tika email karanna puluvandha? </t>
   </si>
   <si>
-    <t xml:space="preserve">Mr. පෙරේරා, මට අඩ office එන්න පරක්කු වෙනවා. මොකද bus eke ගොඩක් සෙනග , හොදටම traffic බත්තරමුල්ල හටියේ. meeting එක පටන් ගන්න කලින් මම එනවා. මට documents ටික email කරන්න පුලුවන්ද? </t>
-  </si>
-  <si>
     <t>Mata assignment ek ivara karanna thava dhavas dhekayi thiyenne. oyaa free nam mata udhav karanna puluvandha? api hat library eke set vela discuss karamu. please mata call ekak ganna. heta ena velaava kathaa kara ganna.</t>
   </si>
   <si>
-    <t>මට assignment එක් ඉවර කරන්න තව දවස් දෙකයි තියෙන්නෙ. ඔයා free නම් මට උදව් කරන්න පුලුවන්ද? අපි හට library eke සෙට් වෙල discuss කරමු. please මට call එකක් ගන්න. හෙට එන වෙලාව කතා කර ගන්න</t>
-  </si>
-  <si>
-    <t>SuBha sandyavak wavaa!</t>
-  </si>
-  <si>
     <t>සුභ සන්ධ්‍යාවක් වවා!</t>
   </si>
   <si>
-    <t>mama ad iskoolayee program ekakata giyaa haebaeyi mama aavee raee velaa.</t>
-  </si>
-  <si>
-    <t>මම අඩ ඉස්කෝලයේ program එකකට ගියා හැබැයි මම ආවේ රෑ වෙලා.</t>
-  </si>
-  <si>
-    <t>මම් ගෙදර යනවා.
-ඔයා එනවද</t>
-  </si>
-  <si>
     <t>api passee katha karmu. Maht  hodatama vahinava saha goravanavaa. mata thaniyama gedhara inna tikak Bhaya hithenavaa. mata dhaen badagini nisaa mama kussiyata yanavaa monava hari kanna. vassa adu unaama mama oyaata gannam.</t>
   </si>
   <si>
-    <t>අපි පස්සේ කතා කරමු. මහට හොඳටම වහිනවා සහ ගොරවනවා. මට තනියම ගෙදර ඉන්න ටිකක් භය හිතෙනවා. මට දැන් බඩගිනි නිසා මම කුස්සියට යනවා මොනව හරි කන්න. වැස්ස අඩු උනාම මම ඔයාට ගන්නම්.</t>
-  </si>
-  <si>
     <t>11/11/2025 dhina mama vaedata paminiyee naetha. namuth maagee nopaeminiima salakunu kara nomaetha, ema nisaa mata mee masa sampuurNa padi mudhal labaa dheyi kiyalaa mama hithanavaa. karunaakara mata ee vistharaya hariyata hoyaa gaeniimata upakaara kala hakid?</t>
   </si>
   <si>
-    <t>11/11/2025 දින මම වැඩට පමිණියේ නැත. නමුත් මාගේ නොපැමිණීම සලකුණු කර නොමැත, එම නිසා මට මේ මස සම්පූර්ණ පඩි මුදල් ලබා දෙයි කියලා මම හිතනවා. කරුණාකර මට ඒ විස්තරය හරියට හොයා ගැනීමට උපකාර කල හකිද?</t>
-  </si>
-  <si>
-    <t>මට Facebook account එක් login වෙන්න  බා. ඇයි ද දන්නේ නෑ නේද?</t>
-  </si>
-  <si>
-    <t>mata Facebook account ek login venna  b. Ai da dannee na need?</t>
-  </si>
-  <si>
     <t>mama adha nandalge gedhara yannee. oyath enavadha ehee yanna?</t>
   </si>
   <si>
@@ -532,78 +474,39 @@
     <t>සුපිරියි! අපි දිනුම ලැබුනා.</t>
   </si>
   <si>
-    <t>කසුන් හට ගෙදර යනවලු ඒක නිසා මම අද එයාව බලන්න ආවා</t>
-  </si>
-  <si>
     <t>kasun hat gadara yanawalu eeka nisaa mam ada eyaava balanna aavaa</t>
   </si>
   <si>
     <t>mata one ek denna karunakara. Mama enna  hithan inne?</t>
   </si>
   <si>
-    <t>මට එක් දෙන්න කරුණාකර. මම එන්න හිතන් ඉන්නේ?</t>
-  </si>
-  <si>
     <t>අයුබෝවන් මැචන්! සුභ අලුත් අවුරුද්දක් වේවා!</t>
   </si>
   <si>
     <t>karunakarala mata ek pnnanna</t>
   </si>
   <si>
-    <t>කරුණාකරලා මට එක් පන්නන්න</t>
-  </si>
-  <si>
     <t>හරි මචං එක කරන්නම්. අනේ ඔයාට ගොඩක් thanks!</t>
   </si>
   <si>
-    <t>හරි මැචන් එක කරන්නම්. අනේ ඔයාට ගොඩක් tanks!</t>
-  </si>
-  <si>
     <t>හරි හරි මම් එන්නම් එන්නම්</t>
   </si>
   <si>
     <t>hari hari mm ennam ennam</t>
   </si>
   <si>
-    <t>mama yanawa... oyath enawada? Ani!</t>
-  </si>
-  <si>
-    <t>මම යනවා... ඔයාත් එනවද? අනී!</t>
-  </si>
-  <si>
     <t>ඔයාලගේ WiFi password එක මරු කරාද?</t>
   </si>
   <si>
     <t>oyalage WiFi password eka mru karada?</t>
   </si>
   <si>
-    <t>Rs 500 ක් ඩන්න</t>
-  </si>
-  <si>
     <t>Rs 500 dnn</t>
   </si>
   <si>
-    <t>man oyat yankota kta karannm. oyta enna puluwanda?</t>
-  </si>
-  <si>
-    <t>මන් ඔයාට  යනකොට කට කරන්නම්. ඔයාට එන්න පුලුවන්ද?</t>
-  </si>
-  <si>
     <t>api ad dinner ganna ar resturant ekt yamud?</t>
   </si>
   <si>
-    <t>අපි අඩ dinner ගන්න අර resturant එකට යමුද?</t>
-  </si>
-  <si>
-    <t>very tired නිසා ඒ මම් ගෙදර යනවා</t>
-  </si>
-  <si>
-    <t>feeling very tired ee nisa mam gedara yanawa</t>
-  </si>
-  <si>
-    <t>ෆෝන් අක දෙන්න කියලා මම කිව්වා නිසා එයා එක දුන්නා.</t>
-  </si>
-  <si>
     <t>phone ak denna kiyala mama kiwwa nisa eya eka dunn</t>
   </si>
   <si>
@@ -613,49 +516,10 @@
     <t>ඔයා  ok</t>
   </si>
   <si>
-    <t>ෆෝන් අක දෙන්න</t>
-  </si>
-  <si>
     <t>phone ak denna</t>
   </si>
   <si>
-    <t xml:space="preserve">I mata office ake meeting akk thiyenava so late veyi. </t>
-  </si>
-  <si>
-    <t>මට office අකේ meeting අකක් තියෙනව සො late වෙයි.</t>
-  </si>
-  <si>
-    <t>මම ගෙද\න්‍රයනවා (Note: ඉන් Excel, press Alt + Enter to create තෙ line break between 'ගෙද' and 'ර')</t>
-  </si>
-  <si>
     <t>අපිහෙටඋදේමයමු</t>
-  </si>
-  <si>
-    <t>ඒඒඑපා කියලා මම කියන්නේ නිසා ඔයාට එක තේරුම් ගන්න ඕනි</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">එයා අද කියවනවා වැඩි නැද්ද. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Iskoola Pota"/>
-        <family val="2"/>
-      </rPr>
-      <t>@</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Iskoola Pota"/>
-        <family val="2"/>
-      </rPr>
-      <t>මට නම් අහන් i#දalලා එපා වෙලා</t>
-    </r>
   </si>
   <si>
     <t>Present tense variation</t>
@@ -734,9 +598,6 @@
     <t>Informal spoken style</t>
   </si>
   <si>
-    <t>මගේ bar 10kg ක් අඩු වෙලා, එම නිසා මට doctor බෙහෙත් ලබා දුන්නා</t>
-  </si>
-  <si>
     <t>hari! (oya?) “ann”</t>
   </si>
   <si>
@@ -747,13 +608,288 @@
   </si>
   <si>
     <t xml:space="preserve"> හරි! (ඔයා?) “අන්න"</t>
+  </si>
+  <si>
+    <t>මම් ගෙදර යනවා.
+ඔයා එනවද?</t>
+  </si>
+  <si>
+    <t>apithmakanavaa</t>
+  </si>
+  <si>
+    <t>අපිතමකනවා.</t>
+  </si>
+  <si>
+    <t>අපි පස්සේ කතා කරමු. මහත් හොදටම වහිනවා සහ ගොරවනවා. මට තනියම ගෙදර ඉන්න ටිකක් භය හිතෙනවා. මට දැන් බඩගිනි නිසා මම කුස්සියට යනවා මොනවා හරි කන්න. වැස්ස අඩු උනාම මම ඔයාට ගන්නම්.</t>
+  </si>
+  <si>
+    <t>අපි trip එක Kandy වලට යමුද traffic නිසා යනකොට පරක්කුවෙි ද?</t>
+  </si>
+  <si>
+    <t>මාර්තු මස මට exam එක තියෙනවා</t>
+  </si>
+  <si>
+    <t>11/11/2025 දින මම වැඩට පැමිනියේ නීත. නමුත් මාගේ නොපඑමිණීම සලකුණු කර නොමඇත, එම නිසා මට මේ මාස සම්පූර්ණ පඩි මුදල් ලබා දෙයි කියලා මම හිතනවා. කරුණාකර මට ඊ විස්තරය හරියට හොයා ගැනිමට උපකාර කල හකිඩ්?</t>
+  </si>
+  <si>
+    <t>මගේ බ්රා 10kg ක් අඩු වෙලා, එම නිසා මට ඩොක්ටර් බෙහෙත් ලබා දුන්නා.</t>
+  </si>
+  <si>
+    <t>හට උඩී 8.30 ට office යන්න එන්න</t>
+  </si>
+  <si>
+    <t>Mr. පැරීරයා, මට අද office එන්න පරක්කු වෙනවා. මොකද බස් එකේ ගොඩක් සෙනග , හොදටම traffic බත්තරමුල්ල හැටියෙ. meeting එක පටන් ගන්න කලින් මම එනවා. මට documents ටික email කරන්න පුලුවන්ද?</t>
+  </si>
+  <si>
+    <t>මට assignment එක ඉවර කරන්න තව දවස් දෙකයි තියෙන්නේ. ඔයා free නම් මට උදව් කරන්න පුලුවන්ද? අපි හාට් library එකේ set වෙලා discuss කරමු. please මට call එකක් ගන්න. හෙට එන වෙලාව කතා කර ගන්න.</t>
+  </si>
+  <si>
+    <t>SuBha sandyavak wava!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ම්ම් අද ඉස්කෝලයේ ප්රෝග්රෑම් එක්කට ගියා හැබැයි මම ආවේ රෑ වෙලා.
+</t>
+  </si>
+  <si>
+    <t>mm ad iskolay program ekkata giyaa haebayi mama aavee raee velaa.</t>
+  </si>
+  <si>
+    <t>mt Facebook account ek login wanna  b. Ai da dannee na need?</t>
+  </si>
+  <si>
+    <t>මට Facebook account එක login වන්න බෑ. ඇයි ද දන්නේ නෑ නේද?</t>
+  </si>
+  <si>
+    <t>කසුන් හාට් ගදර යනවලු ඒක නිසා මම් අද එයාව බලන්න ආවා</t>
+  </si>
+  <si>
+    <t>මට ඕනේ එක් දෙන්න කරුණාකර. මම එන්න හිතන් ඉන්නේ?</t>
+  </si>
+  <si>
+    <t>මට ඒක දෙන්න කරුණාකර. මම එන්න හිතන් ඉන්නේ?</t>
+  </si>
+  <si>
+    <t>අයුබෝවන් මැචන්! සුභ අලුත් අවුරුද්දක් වේවේ!</t>
+  </si>
+  <si>
+    <t>කරුණාකරලා මට ඒක පන්නන්න</t>
+  </si>
+  <si>
+    <t>හරි මචං ඒක කරන්නම්. අනේ ඔයාට ගොඩක් තැන්ක්ස්!</t>
+  </si>
+  <si>
+    <t>මම යනවා... ඔයාට එනවද? අනේ !</t>
+  </si>
+  <si>
+    <t>mma ynw... oyt enwda? Ani!</t>
+  </si>
+  <si>
+    <t>මන් ඔයාට යන්කට කතා කරන්නම්. ඔයාට එන්න පුළුවන්ද?</t>
+  </si>
+  <si>
+    <t>mn oyt yankt kta karannm. oyta enna puluwanda?</t>
+  </si>
+  <si>
+    <t>අපි අද dinner ගන්න ආර් resturant එකට යමුද?</t>
+  </si>
+  <si>
+    <t>feeling very tird ඒ නිසා මම ගෙදර යනවා</t>
+  </si>
+  <si>
+    <t>feeling very tird ee nisa mam gedara ynwa</t>
+  </si>
+  <si>
+    <t>Rs 500 ක් දාන්න</t>
+  </si>
+  <si>
+    <t>phone අක් දෙන්න කියලා මම කිව්වා නිසා එයා ඒක දුන්නා</t>
+  </si>
+  <si>
+    <t>phone අක් දෙන්න</t>
+  </si>
+  <si>
+    <t>නොඔ මම කියන්නේ එයාට එහෙම කරන්න එපා කියලා</t>
+  </si>
+  <si>
+    <t>මට office එකේ meeting එකක් තියෙනවා සෝ ලට් වෙයි.</t>
+  </si>
+  <si>
+    <t>I mata office ake meeting akk tiyenwa so lat veyi.</t>
+  </si>
+  <si>
+    <t>&lt;හ්1&gt;Hello&lt;/හ්1&gt;</t>
+  </si>
+  <si>
+    <t>මම ගෙදර යනවා (Note: ඉන් Excel, press Alt + Enter to create the line break between 'gedha' and 'ra')</t>
+  </si>
+  <si>
+    <t>එයා අද කියවනවා වැඩි නැද්ද. @මට නම් අහන් දාලා එපා වෙලා</t>
+  </si>
+  <si>
+    <t>eyaa adha kiyavanavaa vaedi naedhdha. @mt nm ahan i#dhallaa epaa velaa</t>
+  </si>
+  <si>
+    <t>ඒඒඒපා කියලා මම කියන්නේ නිසා ඔයාට ඒක තේරුම් ගන්න ඕනි</t>
+  </si>
+  <si>
+    <t>Evidence or rationale</t>
+  </si>
+  <si>
+    <t>Input with line breaks and question form. Expected to preserve line break formatting (\n) and convert question mark, but actual output has spacing issues.</t>
+  </si>
+  <si>
+    <t>Spaces removed in actual output - system failed to preserve spacing between syllables (තම vs තාම). Missing critical vowel markers.</t>
+  </si>
+  <si>
+    <t>Pronoun conversion error - converted "aya" (that person) to "aaye" (she) instead of maintaining the original meaning. Gender assumption error.</t>
+  </si>
+  <si>
+    <t>Compound sentence with multiple clauses. System altered "Maht" to "Maha" and changed several word forms incorrectly. Complex sentence parsing failure.</t>
+  </si>
+  <si>
+    <t>Mixed English and Sinhala (Teams, WhatsApp, link). Actual output shows different spacing and article handling for English loan words.</t>
+  </si>
+  <si>
+    <t>Question form with English noun "traffic". System incorrectly converted "parakkuwei" to "parakkuwei" - vowel length marker error.</t>
+  </si>
+  <si>
+    <t>Informal spoken style with contraction "mm ee" (I that about). System output shows incorrect consonant doubling (ම්ම්).</t>
+  </si>
+  <si>
+    <t>Technical terms with English acronym CVV. System altered "ATM Card" to "ATM කාඩ්" but then changed "CVV keethaya" to "CVV කීතය" - inconsistent handling</t>
+  </si>
+  <si>
+    <t>Complex long sentence with date and formal tone. Multiple errors: "dhina" to "දින", "noththa" to "නීත", "heyi" to "නීත". Vowel conversion failures.</t>
+  </si>
+  <si>
+    <t>Simple affirmation with casual "eeka hari". Output shows vowel addition error: "ඔව්" to "ඔව්වා".</t>
+  </si>
+  <si>
+    <t>Short responses with quoted words. Quote handling error - system converted English quotes but failed on single letter "Q" handling.</t>
+  </si>
+  <si>
+    <t>Informal style with "magee bra" (my weight). System output shows wrong consonant: "බ්රා" instead of "බර" - critical meaning change.</t>
+  </si>
+  <si>
+    <t>Command with time specification. System output: "හට උඩී" - should be "හෙට උදේ". Time conversion error.</t>
+  </si>
+  <si>
+    <t>Formal request with English names and English words mixed. System incorrectly handled "Mr. pereeraa" to "Mr. පැරීරයා" and changed "eke" handling.</t>
+  </si>
+  <si>
+    <t>Polite request with English word "library" and informal expressions. System output shows inconsistent spacing in "හාට්" (should be "හෙට") and "එකේ" variations.</t>
+  </si>
+  <si>
+    <t>Greeting/wish expression. Output shows vowel length error: "වවා" instead of "වේවා" - lost the emphatic form.</t>
+  </si>
+  <si>
+    <t>Simple sentence with month name. System changed "masa" to "මස" (wrong case marker) instead of "මාසේ".</t>
+  </si>
+  <si>
+    <t>Informal slang with USD currency. System changed "eyaga padiya" to "එයාග පඩිය" - possessive form error with consonant assimilation.</t>
+  </si>
+  <si>
+    <t>School program statement with mixed formal/informal. System output shows double consonant error: "ම්ම්" instead of "මම්".</t>
+  </si>
+  <si>
+    <t>Technical login issue statement. System failed to properly convert "wanna" - output shows spelling variation "වන්න" vs expected "වෙන්න".</t>
+  </si>
+  <si>
+    <t>Personal invitation with proper name "Nandalge". Output shows spelling variation "නන්දලා" vs "නැන්දලා" for the name</t>
+  </si>
+  <si>
+    <t>Informal celebration statement. System removed required vowel marker: "අපි" should remain but shows "අපිට" vs "අපි" conversion issue.</t>
+  </si>
+  <si>
+    <t>Informal narrative about person leaving. Output shows consonant doubling issue "හාට්" instead of "හෙට".</t>
+  </si>
+  <si>
+    <t>Mixed formal/informal about dinner plans. System added space issue between consonants: "කෑම" handling and English word mixing.</t>
+  </si>
+  <si>
+    <t>Polite request for item. System output shows conversion "ඕනේ" which adds extra meaning compared to simple "ඒක".</t>
+  </si>
+  <si>
+    <t>Casual invitation to watch match. System output shows "match එක" vs "මැච්" - inconsistent English term handling.</t>
+  </si>
+  <si>
+    <t>New Year greeting with informal slang. Output shows vowel error: "වේවේ" instead of "වේවා" - wrong emphasis form.</t>
+  </si>
+  <si>
+    <t>Polite request to show something. System output shows "පන්නන්න" vs expected "පෙන්නන්න" - critical vowel letter substitution.</t>
+  </si>
+  <si>
+    <t>Gratitude expression with slang. System converted "thanks" to "තැන්ක්ස්" instead of maintaining English or using "ස්තූතිය".</t>
+  </si>
+  <si>
+    <t>Urgent/repeated statement. System output shows consonant doubling: "මම්" instead of "මම".</t>
+  </si>
+  <si>
+    <t>Informal casual conversation. System changed "ඔයාත්" to "ඔයාට" - wrong case marker applied.</t>
+  </si>
+  <si>
+    <t>Patriotic statement. System removed critical vowel: "ආදරෙයි" vs "ආදරේ" - lost the auxiliary verb form.</t>
+  </si>
+  <si>
+    <t>Conditional polite request. System output shows vowel variation: "පුලුවන්" vs "පුළුවන්ද" - wrong form of auxiliary.</t>
+  </si>
+  <si>
+    <t>Mixed English/Sinhala about tiredness. Output shows missing English word "feeling" in conversion.</t>
+  </si>
+  <si>
+    <t>Dinner suggestion with English word. System output shows article inconsistency "ආර්" vs "අර".</t>
+  </si>
+  <si>
+    <t>Technical question about WiFi. System output shows spelling variation: "මරු" vs "මාරු" - vowel length error.</t>
+  </si>
+  <si>
+    <t>Simple money request. System output shows verb variation: "දාන්න" vs "දෙන්න" - wrong verb form.</t>
+  </si>
+  <si>
+    <t>Narrative explanation. System output shows consonant issue "phone අක්" to maintain English word.</t>
+  </si>
+  <si>
+    <t>Simple action statement with English. System shows "run" not converted, which is correct for English word.</t>
+  </si>
+  <si>
+    <t>Question about location. System output shows word form "ඔයාගෙ school" - English word mixing inconsistency.</t>
+  </si>
+  <si>
+    <t>Informal agreement. System output shows English "ok" not converted, which is acceptable for slang.</t>
+  </si>
+  <si>
+    <t>Casual command with contraction. System output shows "අක්" which seems to be abbreviation handling.</t>
+  </si>
+  <si>
+    <t>Negation statement. System output shows "නොඔ" instead of "නෝ" - wrong consonant class assignment.</t>
+  </si>
+  <si>
+    <t>System credentials and alphanumeric string. Correctly kept as-is since it contains user ID, password, and system codes.</t>
+  </si>
+  <si>
+    <t>Mixed English and Sinhala in formal context. System changed "So lat veyi" handling - English word integration failure.</t>
+  </si>
+  <si>
+    <t>HTML markup handling. System incorrectly converted HTML tags "&lt;h1&gt;" to "&lt;හ්1&gt;" - should leave markup unchanged.</t>
+  </si>
+  <si>
+    <t>Input with manual line break instruction. Note indicates proper handling requires Alt+Enter for line breaks in Excel.</t>
+  </si>
+  <si>
+    <t>Text with special character and symbol (@). System mishandled email-like format and special character processing.</t>
+  </si>
+  <si>
+    <t>Continuous text without spaces. System correctly returned as-is since input cannot be reliably parsed without spacing.</t>
+  </si>
+  <si>
+    <t>Repeated character emphasis pattern. System output shows handling of repetition: "ඒඒඒපා" which maintains the repetitive emphasis.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -806,6 +942,12 @@
       <i/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -916,7 +1058,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -925,42 +1067,45 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1247,9 +1392,9 @@
   <cols>
     <col min="1" max="1" width="13.6328125" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="53.6328125" customWidth="1"/>
-    <col min="4" max="4" width="67.36328125" customWidth="1"/>
-    <col min="5" max="5" width="48.54296875" customWidth="1"/>
+    <col min="3" max="3" width="43.54296875" customWidth="1"/>
+    <col min="4" max="4" width="42.6328125" customWidth="1"/>
+    <col min="5" max="5" width="36.6328125" customWidth="1"/>
     <col min="6" max="6" width="20.453125" customWidth="1"/>
     <col min="7" max="7" width="45.08984375" customWidth="1"/>
     <col min="8" max="8" width="61.6328125" customWidth="1"/>
@@ -1275,39 +1420,43 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="H1" s="3"/>
+        <v>167</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="2" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="H2" s="4"/>
+      <c r="E2" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
-      <c r="D3" s="10"/>
+      <c r="D3" s="12"/>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
@@ -1317,7 +1466,7 @@
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
-      <c r="D4" s="10"/>
+      <c r="D4" s="12"/>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -1327,41 +1476,43 @@
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
-      <c r="D5" s="11"/>
+      <c r="D5" s="13"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="C6" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="H6" s="4"/>
+      <c r="E6" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
-      <c r="D7" s="10"/>
+      <c r="D7" s="12"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -1371,7 +1522,7 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
-      <c r="D8" s="10"/>
+      <c r="D8" s="12"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
@@ -1381,41 +1532,43 @@
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
-      <c r="D9" s="11"/>
+      <c r="D9" s="13"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="H10" s="4"/>
+      <c r="F10" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
-      <c r="D11" s="10"/>
+      <c r="D11" s="12"/>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
@@ -1425,7 +1578,7 @@
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
-      <c r="D12" s="10"/>
+      <c r="D12" s="12"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
@@ -1435,41 +1588,43 @@
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
-      <c r="D13" s="11"/>
+      <c r="D13" s="13"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="D14" s="15" t="s">
+      <c r="C14" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="D14" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="H14" s="4"/>
+      <c r="E14" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
-      <c r="D15" s="10"/>
+      <c r="D15" s="12"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
@@ -1479,7 +1634,7 @@
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
-      <c r="D16" s="10"/>
+      <c r="D16" s="12"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
@@ -1489,35 +1644,37 @@
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
-      <c r="D17" s="11"/>
+      <c r="D17" s="13"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
     </row>
     <row r="18" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H18" s="4"/>
+      <c r="E18" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5"/>
@@ -1550,28 +1707,30 @@
       <c r="H21" s="6"/>
     </row>
     <row r="22" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="H22" s="4"/>
+      <c r="E22" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
@@ -1604,28 +1763,30 @@
       <c r="H25" s="6"/>
     </row>
     <row r="26" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H26" s="4"/>
+      <c r="E26" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
@@ -1658,28 +1819,30 @@
       <c r="H29" s="6"/>
     </row>
     <row r="30" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H30" s="4"/>
+      <c r="F30" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
@@ -1712,28 +1875,30 @@
       <c r="H33" s="6"/>
     </row>
     <row r="34" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D34" s="4" t="s">
+      <c r="C34" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E34" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H34" s="4"/>
+      <c r="E34" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="35" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5"/>
@@ -1766,28 +1931,30 @@
       <c r="H37" s="6"/>
     </row>
     <row r="38" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="13" t="s">
+      <c r="A38" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C38" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="D38" s="16" t="s">
+      <c r="C38" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E38" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="H38" s="4"/>
+      <c r="E38" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="39" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5"/>
@@ -1820,28 +1987,30 @@
       <c r="H41" s="6"/>
     </row>
     <row r="42" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="D42" s="4" t="s">
+      <c r="C42" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="D42" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E42" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H42" s="4"/>
+      <c r="E42" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="43" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5"/>
@@ -1874,28 +2043,30 @@
       <c r="H45" s="6"/>
     </row>
     <row r="46" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="B46" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="D46" s="4" t="s">
+      <c r="C46" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="D46" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E46" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H46" s="4"/>
+      <c r="E46" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="47" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5"/>
@@ -1928,28 +2099,30 @@
       <c r="H49" s="6"/>
     </row>
     <row r="50" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A50" s="13" t="s">
+      <c r="A50" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="C50" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="D50" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E50" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H50" s="4"/>
+      <c r="E50" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="51" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5"/>
@@ -1982,28 +2155,30 @@
       <c r="H53" s="6"/>
     </row>
     <row r="54" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A54" s="13" t="s">
+      <c r="A54" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C54" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="D54" s="18" t="s">
+      <c r="C54" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D54" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E54" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H54" s="4"/>
+      <c r="E54" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H54" s="7" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="55" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5"/>
@@ -2036,28 +2211,30 @@
       <c r="H57" s="6"/>
     </row>
     <row r="58" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A58" s="13" t="s">
+      <c r="A58" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="B58" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C58" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="D58" s="4" t="s">
+      <c r="C58" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D58" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E58" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H58" s="4"/>
+      <c r="E58" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="59" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5"/>
@@ -2090,28 +2267,30 @@
       <c r="H61" s="6"/>
     </row>
     <row r="62" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A62" s="13" t="s">
+      <c r="A62" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="B62" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C62" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="D62" s="4" t="s">
+      <c r="C62" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D62" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="E62" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="F62" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="H62" s="4"/>
+      <c r="E62" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="F62" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G62" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="H62" s="7" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="63" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A63" s="5"/>
@@ -2144,28 +2323,30 @@
       <c r="H65" s="6"/>
     </row>
     <row r="66" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A66" s="13" t="s">
+      <c r="A66" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B66" s="8" t="s">
+      <c r="B66" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C66" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="D66" s="4" t="s">
+      <c r="C66" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D66" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E66" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="F66" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="H66" s="4"/>
+      <c r="E66" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="H66" s="7" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="67" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5"/>
@@ -2198,28 +2379,30 @@
       <c r="H69" s="6"/>
     </row>
     <row r="70" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A70" s="13" t="s">
+      <c r="A70" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B70" s="8" t="s">
+      <c r="B70" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="C70" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D70" s="4" t="s">
+      <c r="D70" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="E70" s="4" t="s">
+      <c r="E70" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F70" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G70" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H70" s="4"/>
+      <c r="F70" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G70" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H70" s="7" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="71" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5"/>
@@ -2252,28 +2435,30 @@
       <c r="H73" s="6"/>
     </row>
     <row r="74" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A74" s="13" t="s">
+      <c r="A74" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B74" s="8" t="s">
+      <c r="B74" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C74" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="D74" s="4" t="s">
+      <c r="C74" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D74" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E74" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="F74" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G74" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H74" s="4"/>
+      <c r="E74" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="F74" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G74" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H74" s="7" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="75" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5"/>
@@ -2306,28 +2491,30 @@
       <c r="H77" s="6"/>
     </row>
     <row r="78" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A78" s="13" t="s">
+      <c r="A78" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B78" s="8" t="s">
+      <c r="B78" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C78" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="D78" s="4" t="s">
+      <c r="C78" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="D78" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E78" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="F78" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G78" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="H78" s="4"/>
+      <c r="E78" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="F78" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="H78" s="7" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="79" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5"/>
@@ -2360,28 +2547,30 @@
       <c r="H81" s="6"/>
     </row>
     <row r="82" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A82" s="13" t="s">
+      <c r="A82" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B82" s="8" t="s">
+      <c r="B82" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C82" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="D82" s="4" t="s">
+      <c r="C82" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="D82" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E82" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="F82" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G82" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="H82" s="4"/>
+      <c r="E82" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G82" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H82" s="7" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="83" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A83" s="5"/>
@@ -2414,28 +2603,30 @@
       <c r="H85" s="6"/>
     </row>
     <row r="86" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A86" s="13" t="s">
+      <c r="A86" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B86" s="8" t="s">
+      <c r="B86" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C86" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="D86" s="4" t="s">
+      <c r="C86" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="D86" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E86" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="F86" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G86" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H86" s="4"/>
+      <c r="E86" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="F86" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G86" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="H86" s="7" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="87" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5"/>
@@ -2468,28 +2659,30 @@
       <c r="H89" s="6"/>
     </row>
     <row r="90" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A90" s="13" t="s">
+      <c r="A90" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B90" s="8" t="s">
+      <c r="B90" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C90" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="D90" s="4" t="s">
+      <c r="C90" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D90" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E90" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F90" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G90" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H90" s="4"/>
+      <c r="E90" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F90" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G90" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H90" s="7" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="91" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A91" s="5"/>
@@ -2522,28 +2715,30 @@
       <c r="H93" s="6"/>
     </row>
     <row r="94" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A94" s="13" t="s">
+      <c r="A94" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B94" s="8" t="s">
+      <c r="B94" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="C94" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D94" s="4" t="s">
+      <c r="D94" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E94" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F94" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G94" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="H94" s="4"/>
+      <c r="E94" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F94" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="H94" s="7" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="95" spans="1:8" ht="15.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5"/>
@@ -2576,28 +2771,30 @@
       <c r="H97" s="6"/>
     </row>
     <row r="98" spans="1:8" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A98" s="13" t="s">
+      <c r="A98" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B98" s="8" t="s">
+      <c r="B98" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C98" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D98" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="E98" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="F98" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G98" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="H98" s="4"/>
+      <c r="C98" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E98" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="F98" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G98" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H98" s="7" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="99" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A99" s="5"/>
@@ -2630,28 +2827,30 @@
       <c r="H101" s="6"/>
     </row>
     <row r="102" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A102" s="13" t="s">
+      <c r="A102" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C102" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B102" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C102" s="7" t="s">
+      <c r="D102" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D102" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E102" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F102" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G102" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="H102" s="4"/>
+      <c r="E102" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F102" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G102" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H102" s="7" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="103" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A103" s="5"/>
@@ -2684,28 +2883,30 @@
       <c r="H105" s="6"/>
     </row>
     <row r="106" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A106" s="13" t="s">
+      <c r="A106" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C106" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B106" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C106" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D106" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E106" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="F106" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G106" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="H106" s="4"/>
+      <c r="D106" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E106" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="F106" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G106" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H106" s="7" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="107" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A107" s="5"/>
@@ -2738,28 +2939,30 @@
       <c r="H109" s="6"/>
     </row>
     <row r="110" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A110" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="B110" s="8" t="s">
+      <c r="A110" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B110" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C110" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="D110" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E110" s="4" t="s">
+      <c r="C110" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D110" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E110" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="F110" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G110" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="F110" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G110" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="H110" s="4"/>
+      <c r="H110" s="7" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="111" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A111" s="5"/>
@@ -2792,28 +2995,30 @@
       <c r="H113" s="6"/>
     </row>
     <row r="114" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A114" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="B114" s="8" t="s">
+      <c r="A114" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B114" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C114" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D114" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="E114" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="F114" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G114" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="H114" s="4"/>
+      <c r="C114" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E114" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F114" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G114" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="H114" s="7" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="115" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A115" s="5"/>
@@ -2846,28 +3051,30 @@
       <c r="H117" s="6"/>
     </row>
     <row r="118" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A118" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="B118" s="8" t="s">
+      <c r="A118" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B118" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C118" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="D118" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E118" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="F118" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G118" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H118" s="4"/>
+      <c r="C118" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E118" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="F118" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G118" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="H118" s="7" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="119" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A119" s="5"/>
@@ -2900,28 +3107,30 @@
       <c r="H121" s="6"/>
     </row>
     <row r="122" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A122" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="B122" s="8" t="s">
+      <c r="A122" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B122" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C122" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="D122" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E122" s="4" t="s">
+      <c r="C122" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D122" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E122" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="F122" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G122" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="F122" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G122" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="H122" s="4"/>
+      <c r="H122" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="123" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A123" s="5"/>
@@ -2954,28 +3163,30 @@
       <c r="H125" s="6"/>
     </row>
     <row r="126" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A126" s="13" t="s">
+      <c r="A126" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D126" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B126" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C126" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D126" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E126" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="F126" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G126" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="H126" s="4"/>
+      <c r="E126" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F126" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G126" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="H126" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="127" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A127" s="5"/>
@@ -3008,28 +3219,30 @@
       <c r="H129" s="6"/>
     </row>
     <row r="130" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A130" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="B130" s="8" t="s">
+      <c r="A130" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B130" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C130" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="D130" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="E130" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="F130" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G130" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="H130" s="4"/>
+      <c r="C130" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="D130" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E130" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="F130" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G130" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="H130" s="7" t="s">
+        <v>262</v>
+      </c>
     </row>
     <row r="131" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A131" s="5"/>
@@ -3062,28 +3275,30 @@
       <c r="H133" s="6"/>
     </row>
     <row r="134" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A134" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="B134" s="8" t="s">
+      <c r="A134" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B134" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C134" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="D134" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="E134" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="F134" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G134" s="4" t="s">
+      <c r="C134" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D134" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E134" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="H134" s="4"/>
+      <c r="F134" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G134" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="H134" s="7" t="s">
+        <v>264</v>
+      </c>
     </row>
     <row r="135" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A135" s="5"/>
@@ -3116,28 +3331,30 @@
       <c r="H137" s="6"/>
     </row>
     <row r="138" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A138" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="B138" s="8" t="s">
+      <c r="A138" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B138" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C138" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="D138" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E138" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="F138" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G138" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="H138" s="4"/>
+      <c r="C138" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="D138" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E138" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="F138" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G138" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="H138" s="7" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="139" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A139" s="5"/>
@@ -3170,28 +3387,30 @@
       <c r="H141" s="6"/>
     </row>
     <row r="142" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A142" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="B142" s="8" t="s">
+      <c r="A142" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B142" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C142" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="D142" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="E142" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="F142" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G142" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="H142" s="4"/>
+      <c r="C142" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D142" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E142" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="F142" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G142" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="H142" s="7" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="143" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A143" s="5"/>
@@ -3224,28 +3443,30 @@
       <c r="H145" s="6"/>
     </row>
     <row r="146" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A146" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="B146" s="8" t="s">
+      <c r="A146" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B146" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C146" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="D146" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="E146" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="F146" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G146" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H146" s="4"/>
+      <c r="C146" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D146" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E146" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="F146" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G146" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H146" s="7" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="147" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A147" s="5"/>
@@ -3278,28 +3499,30 @@
       <c r="H149" s="6"/>
     </row>
     <row r="150" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A150" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="B150" s="8" t="s">
+      <c r="A150" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B150" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C150" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="D150" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="E150" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="F150" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G150" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H150" s="4"/>
+      <c r="C150" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="D150" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E150" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F150" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G150" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H150" s="7" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="151" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A151" s="5"/>
@@ -3332,28 +3555,30 @@
       <c r="H153" s="6"/>
     </row>
     <row r="154" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A154" s="13" t="s">
+      <c r="A154" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C154" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D154" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B154" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C154" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D154" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="E154" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="F154" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G154" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H154" s="4"/>
+      <c r="E154" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F154" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G154" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H154" s="7" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="155" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A155" s="5"/>
@@ -3386,28 +3611,30 @@
       <c r="H157" s="6"/>
     </row>
     <row r="158" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A158" s="13" t="s">
+      <c r="A158" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D158" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B158" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C158" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="D158" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E158" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="F158" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G158" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="H158" s="4"/>
+      <c r="E158" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F158" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G158" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="H158" s="7" t="s">
+        <v>269</v>
+      </c>
     </row>
     <row r="159" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A159" s="5"/>
@@ -3440,28 +3667,30 @@
       <c r="H161" s="6"/>
     </row>
     <row r="162" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A162" s="13" t="s">
+      <c r="A162" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C162" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D162" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B162" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C162" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="D162" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E162" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F162" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G162" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H162" s="4"/>
+      <c r="E162" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="F162" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G162" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="H162" s="7" t="s">
+        <v>270</v>
+      </c>
     </row>
     <row r="163" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A163" s="5"/>
@@ -3494,28 +3723,30 @@
       <c r="H165" s="6"/>
     </row>
     <row r="166" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A166" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B166" s="8" t="s">
+      <c r="A166" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B166" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C166" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="D166" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="E166" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="F166" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G166" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H166" s="4"/>
+      <c r="C166" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D166" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E166" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F166" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G166" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H166" s="7" t="s">
+        <v>271</v>
+      </c>
     </row>
     <row r="167" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A167" s="5"/>
@@ -3548,26 +3779,30 @@
       <c r="H169" s="6"/>
     </row>
     <row r="170" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A170" s="13" t="s">
+      <c r="A170" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B170" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C170" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D170" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B170" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C170" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="D170" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="E170" s="4"/>
-      <c r="F170" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G170" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H170" s="4"/>
+      <c r="E170" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="F170" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G170" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H170" s="7" t="s">
+        <v>272</v>
+      </c>
     </row>
     <row r="171" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A171" s="5"/>
@@ -3600,28 +3835,30 @@
       <c r="H173" s="6"/>
     </row>
     <row r="174" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A174" s="13" t="s">
+      <c r="A174" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C174" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D174" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B174" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C174" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="D174" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="E174" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="F174" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G174" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="H174" s="4"/>
+      <c r="E174" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="F174" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G174" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="H174" s="7" t="s">
+        <v>273</v>
+      </c>
     </row>
     <row r="175" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A175" s="5"/>
@@ -3654,28 +3891,30 @@
       <c r="H177" s="6"/>
     </row>
     <row r="178" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A178" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="B178" s="8" t="s">
+      <c r="A178" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B178" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C178" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="D178" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="E178" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="F178" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G178" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="H178" s="4"/>
+      <c r="C178" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="D178" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E178" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F178" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G178" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="H178" s="7" t="s">
+        <v>274</v>
+      </c>
     </row>
     <row r="179" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A179" s="5"/>
@@ -3708,28 +3947,30 @@
       <c r="H181" s="6"/>
     </row>
     <row r="182" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A182" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B182" s="8" t="s">
+      <c r="A182" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B182" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C182" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D182" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E182" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="F182" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G182" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="H182" s="4"/>
+      <c r="C182" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="D182" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E182" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="F182" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G182" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="H182" s="7" t="s">
+        <v>275</v>
+      </c>
     </row>
     <row r="183" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A183" s="5"/>
@@ -3762,28 +4003,30 @@
       <c r="H185" s="6"/>
     </row>
     <row r="186" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A186" s="13" t="s">
+      <c r="A186" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C186" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D186" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B186" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C186" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D186" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="E186" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F186" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G186" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H186" s="4"/>
+      <c r="E186" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="F186" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G186" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H186" s="7" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="187" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A187" s="5"/>
@@ -3816,28 +4059,30 @@
       <c r="H189" s="6"/>
     </row>
     <row r="190" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A190" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="B190" s="8" t="s">
+      <c r="A190" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B190" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C190" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="D190" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E190" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="F190" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G190" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="H190" s="4"/>
+      <c r="C190" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="D190" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E190" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F190" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G190" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="H190" s="7" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="191" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A191" s="5"/>
@@ -3870,28 +4115,30 @@
       <c r="H193" s="6"/>
     </row>
     <row r="194" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A194" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="B194" s="8" t="s">
+      <c r="A194" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B194" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C194" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D194" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E194" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="F194" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G194" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="H194" s="4"/>
+      <c r="C194" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D194" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E194" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="F194" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G194" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="H194" s="7" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="195" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A195" s="5"/>
@@ -3924,28 +4171,30 @@
       <c r="H197" s="6"/>
     </row>
     <row r="198" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A198" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="B198" s="8" t="s">
+      <c r="A198" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B198" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C198" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="D198" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="E198" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="F198" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G198" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="H198" s="4"/>
+      <c r="C198" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D198" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E198" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="F198" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G198" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="H198" s="7" t="s">
+        <v>279</v>
+      </c>
     </row>
     <row r="199" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A199" s="5"/>
@@ -3978,7 +4227,7 @@
       <c r="H201" s="6"/>
     </row>
     <row r="202" spans="1:8" ht="15.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A202" s="13"/>
+      <c r="A202" s="8"/>
     </row>
     <row r="203" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A203" s="5"/>
@@ -3992,6 +4241,383 @@
     <row r="206" spans="1:8" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="401">
+    <mergeCell ref="H182:H185"/>
+    <mergeCell ref="H186:H189"/>
+    <mergeCell ref="H190:H193"/>
+    <mergeCell ref="H194:H197"/>
+    <mergeCell ref="H198:H201"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="H154:H157"/>
+    <mergeCell ref="H158:H161"/>
+    <mergeCell ref="H162:H165"/>
+    <mergeCell ref="H166:H169"/>
+    <mergeCell ref="H170:H173"/>
+    <mergeCell ref="H174:H177"/>
+    <mergeCell ref="H178:H181"/>
+    <mergeCell ref="H110:H113"/>
+    <mergeCell ref="H114:H117"/>
+    <mergeCell ref="H118:H121"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="H130:H133"/>
+    <mergeCell ref="H134:H137"/>
+    <mergeCell ref="H138:H141"/>
+    <mergeCell ref="H142:H145"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="H90:H93"/>
+    <mergeCell ref="H94:H97"/>
+    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="H106:H109"/>
+    <mergeCell ref="G174:G177"/>
+    <mergeCell ref="G178:G181"/>
+    <mergeCell ref="G182:G185"/>
+    <mergeCell ref="G186:G189"/>
+    <mergeCell ref="G190:G193"/>
+    <mergeCell ref="G194:G197"/>
+    <mergeCell ref="G198:G201"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="G138:G141"/>
+    <mergeCell ref="G142:G145"/>
+    <mergeCell ref="G146:G149"/>
+    <mergeCell ref="G150:G153"/>
+    <mergeCell ref="G154:G157"/>
+    <mergeCell ref="G158:G161"/>
+    <mergeCell ref="G162:G165"/>
+    <mergeCell ref="G166:G169"/>
+    <mergeCell ref="G170:G173"/>
+    <mergeCell ref="G102:G105"/>
+    <mergeCell ref="G106:G109"/>
+    <mergeCell ref="G110:G113"/>
+    <mergeCell ref="G114:G117"/>
+    <mergeCell ref="G118:G121"/>
+    <mergeCell ref="G122:G125"/>
+    <mergeCell ref="G126:G129"/>
+    <mergeCell ref="G130:G133"/>
+    <mergeCell ref="G134:G137"/>
+    <mergeCell ref="G66:G69"/>
+    <mergeCell ref="G70:G73"/>
+    <mergeCell ref="G74:G77"/>
+    <mergeCell ref="G78:G81"/>
+    <mergeCell ref="G82:G85"/>
+    <mergeCell ref="G86:G89"/>
+    <mergeCell ref="G90:G93"/>
+    <mergeCell ref="G94:G97"/>
+    <mergeCell ref="G98:G101"/>
+    <mergeCell ref="G34:G37"/>
+    <mergeCell ref="G38:G41"/>
+    <mergeCell ref="G42:G45"/>
+    <mergeCell ref="G46:G49"/>
+    <mergeCell ref="G50:G53"/>
+    <mergeCell ref="G54:G57"/>
+    <mergeCell ref="G58:G61"/>
+    <mergeCell ref="G62:G65"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="G6:G9"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="G14:G17"/>
+    <mergeCell ref="G18:G21"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="G26:G29"/>
+    <mergeCell ref="G30:G33"/>
+    <mergeCell ref="C190:C193"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="C158:C161"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="E190:E193"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="E162:E165"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="F86:F89"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="C90:C93"/>
+    <mergeCell ref="D122:D125"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="D162:D165"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="C110:C113"/>
+    <mergeCell ref="C150:C153"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="D86:D89"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="A202:A205"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="E194:E197"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="A198:A201"/>
+    <mergeCell ref="F194:F197"/>
+    <mergeCell ref="C198:C201"/>
+    <mergeCell ref="F122:F125"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A190:A193"/>
+    <mergeCell ref="F186:F189"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="C138:C141"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="B174:B177"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="E198:E201"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="A154:A157"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="E74:E77"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="E154:E157"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="F106:F109"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="C182:C185"/>
+    <mergeCell ref="E182:E185"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="E118:E121"/>
+    <mergeCell ref="D106:D109"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B158:B161"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="E26:E29"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="D198:D201"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="F198:F201"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D174:D177"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="F174:F177"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="D126:D129"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="E94:E97"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A194:A197"/>
     <mergeCell ref="B38:B41"/>
     <mergeCell ref="D150:D153"/>
     <mergeCell ref="F110:F113"/>
@@ -4016,384 +4642,8 @@
     <mergeCell ref="A38:A41"/>
     <mergeCell ref="A130:A133"/>
     <mergeCell ref="A82:A85"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="D198:D201"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="F198:F201"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D174:D177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="F174:F177"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="D126:D129"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="E94:E97"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="E26:E29"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="E74:E77"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="B118:B121"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="E154:E157"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="D170:D173"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="A154:A157"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="B174:B177"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="E106:E109"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="E198:E201"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="C182:C185"/>
-    <mergeCell ref="E182:E185"/>
-    <mergeCell ref="F106:F109"/>
-    <mergeCell ref="A190:A193"/>
-    <mergeCell ref="F186:F189"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="C166:C169"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="C138:C141"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="C118:C121"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="D106:D109"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="C194:C197"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="A202:A205"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E194:E197"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="A198:A201"/>
-    <mergeCell ref="F194:F197"/>
-    <mergeCell ref="C198:C201"/>
-    <mergeCell ref="F122:F125"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="D162:D165"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="C110:C113"/>
-    <mergeCell ref="C150:C153"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="D86:D89"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="F86:F89"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="C90:C93"/>
-    <mergeCell ref="D122:D125"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="C190:C193"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="F170:F173"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="E134:E137"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="F54:F57"/>
-    <mergeCell ref="C158:C161"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="E162:E165"/>
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="G6:G9"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="G14:G17"/>
-    <mergeCell ref="G18:G21"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="G26:G29"/>
-    <mergeCell ref="G30:G33"/>
-    <mergeCell ref="G34:G37"/>
-    <mergeCell ref="G38:G41"/>
-    <mergeCell ref="G42:G45"/>
-    <mergeCell ref="G46:G49"/>
-    <mergeCell ref="G50:G53"/>
-    <mergeCell ref="G54:G57"/>
-    <mergeCell ref="G58:G61"/>
-    <mergeCell ref="G62:G65"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="G66:G69"/>
-    <mergeCell ref="G70:G73"/>
-    <mergeCell ref="G74:G77"/>
-    <mergeCell ref="G78:G81"/>
-    <mergeCell ref="G82:G85"/>
-    <mergeCell ref="G86:G89"/>
-    <mergeCell ref="G90:G93"/>
-    <mergeCell ref="G94:G97"/>
-    <mergeCell ref="G98:G101"/>
-    <mergeCell ref="G102:G105"/>
-    <mergeCell ref="G106:G109"/>
-    <mergeCell ref="G110:G113"/>
-    <mergeCell ref="G114:G117"/>
-    <mergeCell ref="G118:G121"/>
-    <mergeCell ref="G122:G125"/>
-    <mergeCell ref="G126:G129"/>
-    <mergeCell ref="G130:G133"/>
-    <mergeCell ref="G134:G137"/>
-    <mergeCell ref="G138:G141"/>
-    <mergeCell ref="G142:G145"/>
-    <mergeCell ref="G146:G149"/>
-    <mergeCell ref="G150:G153"/>
-    <mergeCell ref="G154:G157"/>
-    <mergeCell ref="G158:G161"/>
-    <mergeCell ref="G162:G165"/>
-    <mergeCell ref="G166:G169"/>
-    <mergeCell ref="G170:G173"/>
-    <mergeCell ref="G174:G177"/>
-    <mergeCell ref="G178:G181"/>
-    <mergeCell ref="G182:G185"/>
-    <mergeCell ref="G186:G189"/>
-    <mergeCell ref="G190:G193"/>
-    <mergeCell ref="G194:G197"/>
-    <mergeCell ref="G198:G201"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="H22:H25"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="H46:H49"/>
-    <mergeCell ref="H50:H53"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="H78:H81"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="H90:H93"/>
-    <mergeCell ref="H94:H97"/>
-    <mergeCell ref="H98:H101"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="H106:H109"/>
-    <mergeCell ref="H110:H113"/>
-    <mergeCell ref="H114:H117"/>
-    <mergeCell ref="H118:H121"/>
-    <mergeCell ref="H122:H125"/>
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="H130:H133"/>
-    <mergeCell ref="H134:H137"/>
-    <mergeCell ref="H138:H141"/>
-    <mergeCell ref="H142:H145"/>
-    <mergeCell ref="H182:H185"/>
-    <mergeCell ref="H186:H189"/>
-    <mergeCell ref="H190:H193"/>
-    <mergeCell ref="H194:H197"/>
-    <mergeCell ref="H198:H201"/>
-    <mergeCell ref="H146:H149"/>
-    <mergeCell ref="H150:H153"/>
-    <mergeCell ref="H154:H157"/>
-    <mergeCell ref="H158:H161"/>
-    <mergeCell ref="H162:H165"/>
-    <mergeCell ref="H166:H169"/>
-    <mergeCell ref="H170:H173"/>
-    <mergeCell ref="H174:H177"/>
-    <mergeCell ref="H178:H181"/>
   </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>